<commit_message>
feat: Add intraday simulation overlay removal functionality and enhance overlay comparison UI
</commit_message>
<xml_diff>
--- a/data/simulated_intraday_PAX.xlsx
+++ b/data/simulated_intraday_PAX.xlsx
@@ -1434,7 +1434,7 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1455,7 +1455,7 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
@@ -1481,7 +1481,7 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -1502,7 +1502,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="M22" t="n">
         <v>0</v>
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -1546,10 +1546,10 @@
         <v>19</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="M23" t="n">
         <v>0</v>
@@ -1575,7 +1575,7 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -1593,10 +1593,10 @@
         <v>31</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="M24" t="n">
         <v>0</v>
@@ -1622,7 +1622,7 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -1640,10 +1640,10 @@
         <v>69</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
@@ -1669,7 +1669,7 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -1687,10 +1687,10 @@
         <v>141</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
@@ -1716,7 +1716,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>288</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1734,10 +1734,10 @@
         <v>236</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="L27" t="n">
-        <v>3</v>
+        <v>397</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
@@ -1763,10 +1763,10 @@
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>8</v>
+        <v>481</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1781,13 +1781,13 @@
         <v>293</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="L28" t="n">
-        <v>12</v>
+        <v>662</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
@@ -1810,10 +1810,10 @@
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>19</v>
+        <v>664</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -1828,13 +1828,13 @@
         <v>302</v>
       </c>
       <c r="K29" t="n">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="L29" t="n">
-        <v>27</v>
+        <v>914</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
@@ -1857,10 +1857,10 @@
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>37</v>
+        <v>701</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>196</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -1875,13 +1875,13 @@
         <v>196</v>
       </c>
       <c r="K30" t="n">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="L30" t="n">
-        <v>51</v>
+        <v>965</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>269</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
@@ -1904,10 +1904,10 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>73</v>
+        <v>571</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>274</v>
       </c>
       <c r="G31" t="n">
         <v>27</v>
@@ -1922,13 +1922,13 @@
         <v>156</v>
       </c>
       <c r="K31" t="n">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="L31" t="n">
-        <v>100</v>
+        <v>784</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>377</v>
       </c>
       <c r="N31" t="n">
         <v>43</v>
@@ -1951,10 +1951,10 @@
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>148</v>
+        <v>449</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="G32" t="n">
         <v>41</v>
@@ -1969,13 +1969,13 @@
         <v>93</v>
       </c>
       <c r="K32" t="n">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="L32" t="n">
-        <v>204</v>
+        <v>618</v>
       </c>
       <c r="M32" t="n">
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="N32" t="n">
         <v>64</v>
@@ -1998,10 +1998,10 @@
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>288</v>
+        <v>345</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="G33" t="n">
         <v>45</v>
@@ -2016,13 +2016,13 @@
         <v>4</v>
       </c>
       <c r="K33" t="n">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="L33" t="n">
-        <v>397</v>
+        <v>474</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>227</v>
       </c>
       <c r="N33" t="n">
         <v>71</v>
@@ -2045,10 +2045,10 @@
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>481</v>
+        <v>131</v>
       </c>
       <c r="F34" t="n">
-        <v>11</v>
+        <v>221</v>
       </c>
       <c r="G34" t="n">
         <v>83</v>
@@ -2063,13 +2063,13 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="L34" t="n">
-        <v>662</v>
+        <v>180</v>
       </c>
       <c r="M34" t="n">
-        <v>16</v>
+        <v>305</v>
       </c>
       <c r="N34" t="n">
         <v>129</v>
@@ -2092,10 +2092,10 @@
         <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>664</v>
+        <v>8</v>
       </c>
       <c r="F35" t="n">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="G35" t="n">
         <v>70</v>
@@ -2110,13 +2110,13 @@
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="L35" t="n">
-        <v>914</v>
+        <v>12</v>
       </c>
       <c r="M35" t="n">
-        <v>110</v>
+        <v>47</v>
       </c>
       <c r="N35" t="n">
         <v>110</v>
@@ -2139,10 +2139,10 @@
         <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>701</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>196</v>
+        <v>0</v>
       </c>
       <c r="G36" t="n">
         <v>56</v>
@@ -2157,13 +2157,13 @@
         <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>965</v>
+        <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>269</v>
+        <v>0</v>
       </c>
       <c r="N36" t="n">
         <v>87</v>
@@ -2186,10 +2186,10 @@
         <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>571</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>274</v>
+        <v>0</v>
       </c>
       <c r="G37" t="n">
         <v>51</v>
@@ -2204,13 +2204,13 @@
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>784</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>377</v>
+        <v>0</v>
       </c>
       <c r="N37" t="n">
         <v>80</v>
@@ -2233,10 +2233,10 @@
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>449</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>152</v>
+        <v>0</v>
       </c>
       <c r="G38" t="n">
         <v>15</v>
@@ -2251,13 +2251,13 @@
         <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>618</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>208</v>
+        <v>0</v>
       </c>
       <c r="N38" t="n">
         <v>24</v>
@@ -2280,10 +2280,10 @@
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>345</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>165</v>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
         <v>1</v>
@@ -2298,13 +2298,13 @@
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>474</v>
+        <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>227</v>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
         <v>1</v>
@@ -2327,10 +2327,10 @@
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>2086</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
@@ -2345,13 +2345,13 @@
         <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>2868</v>
+        <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>351</v>
+        <v>0</v>
       </c>
       <c r="N40" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat: Enhance intraday PAX simulation with overlay window functionality and UI improvements
</commit_message>
<xml_diff>
--- a/data/simulated_intraday_PAX.xlsx
+++ b/data/simulated_intraday_PAX.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="_overlay_meta" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1378,7 +1379,7 @@
         <v>46155.1875</v>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
@@ -1399,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1425,10 +1426,10 @@
         <v>46155.19791666666</v>
       </c>
       <c r="B21" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -1446,16 +1447,16 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
@@ -1472,16 +1473,16 @@
         <v>46155.20833333334</v>
       </c>
       <c r="B22" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C22" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -1493,16 +1494,16 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
         <v>0</v>
@@ -1519,16 +1520,16 @@
         <v>46155.21875</v>
       </c>
       <c r="B23" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -1540,16 +1541,16 @@
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
         <v>0</v>
@@ -1566,16 +1567,16 @@
         <v>46155.22916666666</v>
       </c>
       <c r="B24" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -1587,10 +1588,10 @@
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1613,16 +1614,16 @@
         <v>46155.23958333334</v>
       </c>
       <c r="B25" t="n">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="C25" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -1634,10 +1635,10 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>141</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1660,16 +1661,16 @@
         <v>46155.25</v>
       </c>
       <c r="B26" t="n">
-        <v>171</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>148</v>
+        <v>119</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -1681,13 +1682,13 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>236</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>141</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
@@ -1707,16 +1708,16 @@
         <v>46155.26041666666</v>
       </c>
       <c r="B27" t="n">
-        <v>213</v>
+        <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>171</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>288</v>
+        <v>231</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1728,13 +1729,13 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>293</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>236</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -1754,19 +1755,19 @@
         <v>46155.27083333334</v>
       </c>
       <c r="B28" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="C28" t="n">
-        <v>213</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>481</v>
+        <v>388</v>
       </c>
       <c r="F28" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1775,19 +1776,19 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>302</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>293</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
@@ -1801,19 +1802,19 @@
         <v>46155.28125</v>
       </c>
       <c r="B29" t="n">
-        <v>143</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>664</v>
+        <v>544</v>
       </c>
       <c r="F29" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -1822,19 +1823,19 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>196</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>302</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
@@ -1848,19 +1849,19 @@
         <v>46155.29166666666</v>
       </c>
       <c r="B30" t="n">
-        <v>113</v>
+        <v>0</v>
       </c>
       <c r="C30" t="n">
-        <v>143</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>701</v>
+        <v>591</v>
       </c>
       <c r="F30" t="n">
-        <v>196</v>
+        <v>153</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -1869,16 +1870,16 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>156</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>196</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>442</v>
+        <v>0</v>
       </c>
       <c r="M30" t="n">
         <v>0</v>
@@ -1895,46 +1896,46 @@
         <v>46155.30208333334</v>
       </c>
       <c r="B31" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>113</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>571</v>
+        <v>509</v>
       </c>
       <c r="F31" t="n">
-        <v>274</v>
+        <v>221</v>
       </c>
       <c r="G31" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>156</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>1007</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="O31" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1942,46 +1943,46 @@
         <v>46155.3125</v>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>449</v>
+        <v>432</v>
       </c>
       <c r="F32" t="n">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="G32" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>133</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>1217</v>
+        <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>313</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>208</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -1992,43 +1993,43 @@
         <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="F33" t="n">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G33" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>1010</v>
+        <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>486</v>
+        <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>271</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -2045,16 +2046,16 @@
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="F34" t="n">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="G34" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
@@ -2063,19 +2064,19 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>936</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>139</v>
+        <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="O34" t="n">
-        <v>201</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -2092,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -2110,19 +2111,19 @@
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>811</v>
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>358</v>
+        <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="O35" t="n">
-        <v>248</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -2145,10 +2146,10 @@
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>155</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -2157,19 +2158,19 @@
         <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>311</v>
+        <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>526</v>
+        <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="O36" t="n">
-        <v>240</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -2192,10 +2193,10 @@
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -2204,19 +2205,19 @@
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="O37" t="n">
-        <v>185</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -2239,10 +2240,10 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
@@ -2260,10 +2261,10 @@
         <v>0</v>
       </c>
       <c r="N38" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="O38" t="n">
-        <v>93</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -2286,10 +2287,10 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -2307,10 +2308,10 @@
         <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O39" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -2357,7 +2358,7 @@
         <v>0</v>
       </c>
       <c r="O40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -5037,6 +5038,114 @@
       </c>
       <c r="O97" t="n">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>StartMinute</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>EndMinute</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>T1_Boarding</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>370</v>
+      </c>
+      <c r="D2" t="n">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>T1_Boarding</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>400</v>
+      </c>
+      <c r="D3" t="n">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>T1_Lounge</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>280</v>
+      </c>
+      <c r="D4" t="n">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>T1_Lounge</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>310</v>
+      </c>
+      <c r="D5" t="n">
+        <v>490</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add impact assessment functionality to intraday PAX simulation and enhance UI elements
</commit_message>
<xml_diff>
--- a/data/simulated_intraday_PAX.xlsx
+++ b/data/simulated_intraday_PAX.xlsx
@@ -1379,7 +1379,7 @@
         <v>46155.1875</v>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
@@ -1426,10 +1426,10 @@
         <v>46155.19791666666</v>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -1473,10 +1473,10 @@
         <v>46155.20833333334</v>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -1520,10 +1520,10 @@
         <v>46155.21875</v>
       </c>
       <c r="B23" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -1567,10 +1567,10 @@
         <v>46155.22916666666</v>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -1614,10 +1614,10 @@
         <v>46155.23958333334</v>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -1661,10 +1661,10 @@
         <v>46155.25</v>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -1708,10 +1708,10 @@
         <v>46155.26041666666</v>
       </c>
       <c r="B27" t="n">
-        <v>0</v>
+        <v>175</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -1755,10 +1755,10 @@
         <v>46155.27083333334</v>
       </c>
       <c r="B28" t="n">
-        <v>0</v>
+        <v>187</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -1802,7 +1802,7 @@
         <v>46155.28125</v>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>132</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
@@ -1849,7 +1849,7 @@
         <v>46155.29166666666</v>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
@@ -1896,7 +1896,7 @@
         <v>46155.30208333334</v>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
@@ -1911,10 +1911,10 @@
         <v>221</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
         <v>46155.3125</v>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
@@ -1958,10 +1958,10 @@
         <v>140</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
@@ -2005,10 +2005,10 @@
         <v>171</v>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -2052,10 +2052,10 @@
         <v>207</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
@@ -2099,10 +2099,10 @@
         <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -2146,10 +2146,10 @@
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>147</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -2193,10 +2193,10 @@
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -5051,7 +5051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5084,14 +5084,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Baggage</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>370</v>
+        <v>420</v>
       </c>
       <c r="D2" t="n">
-        <v>460</v>
+        <v>510</v>
       </c>
     </row>
     <row r="3">
@@ -5102,14 +5102,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Baggage</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="D3" t="n">
-        <v>490</v>
+        <v>540</v>
       </c>
     </row>
     <row r="4">
@@ -5120,11 +5120,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>T1_Lounge</t>
+          <t>T1_Boarding</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>280</v>
+        <v>370</v>
       </c>
       <c r="D4" t="n">
         <v>460</v>
@@ -5138,14 +5138,158 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>T1_Boarding</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>400</v>
+      </c>
+      <c r="D5" t="n">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>T1_Checkin</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>280</v>
+      </c>
+      <c r="D6" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>T1_Checkin</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>310</v>
+      </c>
+      <c r="D7" t="n">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>T1_Immigration</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>420</v>
+      </c>
+      <c r="D8" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>T1_Immigration</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>450</v>
+      </c>
+      <c r="D9" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>T1_Lounge</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C10" t="n">
+        <v>280</v>
+      </c>
+      <c r="D10" t="n">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>T1_Lounge</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>310</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D11" t="n">
         <v>490</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>T1_Security</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>295</v>
+      </c>
+      <c r="D12" t="n">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>T1_Security</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>325</v>
+      </c>
+      <c r="D13" t="n">
+        <v>400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Implement combined flight delay overlay functionality and enhance UI for FTE metrics
</commit_message>
<xml_diff>
--- a/data/simulated_intraday_PAX.xlsx
+++ b/data/simulated_intraday_PAX.xlsx
@@ -1191,7 +1191,7 @@
         <v>46156.14583333334</v>
       </c>
       <c r="B16" t="n">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="C16" t="n">
         <v>-11</v>
@@ -1238,10 +1238,10 @@
         <v>46156.15625</v>
       </c>
       <c r="B17" t="n">
-        <v>-35</v>
+        <v>-40</v>
       </c>
       <c r="C17" t="n">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -1256,10 +1256,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="I17" t="n">
-        <v>-32</v>
+        <v>-34</v>
       </c>
       <c r="J17" t="n">
         <v>-21</v>
@@ -1285,10 +1285,10 @@
         <v>46156.16666666666</v>
       </c>
       <c r="B18" t="n">
-        <v>-72</v>
+        <v>-79</v>
       </c>
       <c r="C18" t="n">
-        <v>-35</v>
+        <v>-40</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -1303,13 +1303,13 @@
         <v>-2</v>
       </c>
       <c r="H18" t="n">
-        <v>-35</v>
+        <v>-40</v>
       </c>
       <c r="I18" t="n">
-        <v>-59</v>
+        <v>-68</v>
       </c>
       <c r="J18" t="n">
-        <v>-32</v>
+        <v>-34</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>-32</v>
+        <v>-34</v>
       </c>
     </row>
     <row r="19">
@@ -1332,10 +1332,10 @@
         <v>46156.17708333334</v>
       </c>
       <c r="B19" t="n">
-        <v>-126</v>
+        <v>-144</v>
       </c>
       <c r="C19" t="n">
-        <v>-72</v>
+        <v>-79</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -1350,13 +1350,13 @@
         <v>-11</v>
       </c>
       <c r="H19" t="n">
-        <v>-72</v>
+        <v>-79</v>
       </c>
       <c r="I19" t="n">
-        <v>-113</v>
+        <v>-130</v>
       </c>
       <c r="J19" t="n">
-        <v>-59</v>
+        <v>-68</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1371,7 +1371,7 @@
         <v>-6</v>
       </c>
       <c r="O19" t="n">
-        <v>-59</v>
+        <v>-68</v>
       </c>
     </row>
     <row r="20">
@@ -1379,10 +1379,10 @@
         <v>46156.1875</v>
       </c>
       <c r="B20" t="n">
-        <v>-247</v>
+        <v>-273</v>
       </c>
       <c r="C20" t="n">
-        <v>-126</v>
+        <v>-144</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -1394,16 +1394,16 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="H20" t="n">
-        <v>-126</v>
+        <v>-144</v>
       </c>
       <c r="I20" t="n">
-        <v>-205</v>
+        <v>-233</v>
       </c>
       <c r="J20" t="n">
-        <v>-113</v>
+        <v>-130</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1418,7 +1418,7 @@
         <v>-21</v>
       </c>
       <c r="O20" t="n">
-        <v>-113</v>
+        <v>-130</v>
       </c>
     </row>
     <row r="21">
@@ -1426,10 +1426,10 @@
         <v>46156.19791666666</v>
       </c>
       <c r="B21" t="n">
-        <v>-331</v>
+        <v>-382</v>
       </c>
       <c r="C21" t="n">
-        <v>-247</v>
+        <v>-273</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -1441,16 +1441,16 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>-35</v>
+        <v>-40</v>
       </c>
       <c r="H21" t="n">
-        <v>-247</v>
+        <v>-273</v>
       </c>
       <c r="I21" t="n">
-        <v>-417</v>
+        <v>-469</v>
       </c>
       <c r="J21" t="n">
-        <v>-205</v>
+        <v>-233</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1462,10 +1462,10 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>-32</v>
+        <v>-34</v>
       </c>
       <c r="O21" t="n">
-        <v>-205</v>
+        <v>-233</v>
       </c>
     </row>
     <row r="22">
@@ -1473,31 +1473,31 @@
         <v>46156.20833333334</v>
       </c>
       <c r="B22" t="n">
-        <v>-99</v>
+        <v>-209</v>
       </c>
       <c r="C22" t="n">
-        <v>-331</v>
+        <v>-382</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>-72</v>
+        <v>-79</v>
       </c>
       <c r="H22" t="n">
-        <v>-331</v>
+        <v>-382</v>
       </c>
       <c r="I22" t="n">
-        <v>-305</v>
+        <v>-398</v>
       </c>
       <c r="J22" t="n">
-        <v>-417</v>
+        <v>-469</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1509,10 +1509,10 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>-59</v>
+        <v>-68</v>
       </c>
       <c r="O22" t="n">
-        <v>-417</v>
+        <v>-469</v>
       </c>
     </row>
     <row r="23">
@@ -1520,46 +1520,46 @@
         <v>46156.21875</v>
       </c>
       <c r="B23" t="n">
-        <v>-23</v>
+        <v>-48</v>
       </c>
       <c r="C23" t="n">
-        <v>-99</v>
+        <v>-209</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>-35</v>
+        <v>-40</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>-126</v>
+        <v>-144</v>
       </c>
       <c r="H23" t="n">
-        <v>-99</v>
+        <v>-209</v>
       </c>
       <c r="I23" t="n">
-        <v>-44</v>
+        <v>-230</v>
       </c>
       <c r="J23" t="n">
-        <v>-305</v>
+        <v>-398</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>-32</v>
+        <v>-34</v>
       </c>
       <c r="M23" t="n">
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>-113</v>
+        <v>-130</v>
       </c>
       <c r="O23" t="n">
-        <v>-305</v>
+        <v>-398</v>
       </c>
     </row>
     <row r="24">
@@ -1567,46 +1567,46 @@
         <v>46156.22916666666</v>
       </c>
       <c r="B24" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="C24" t="n">
-        <v>-23</v>
+        <v>-48</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>-72</v>
+        <v>-79</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>-247</v>
+        <v>-273</v>
       </c>
       <c r="H24" t="n">
-        <v>-23</v>
+        <v>-48</v>
       </c>
       <c r="I24" t="n">
-        <v>97</v>
+        <v>-106</v>
       </c>
       <c r="J24" t="n">
-        <v>-44</v>
+        <v>-230</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>-59</v>
+        <v>-68</v>
       </c>
       <c r="M24" t="n">
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>-205</v>
+        <v>-233</v>
       </c>
       <c r="O24" t="n">
-        <v>-44</v>
+        <v>-230</v>
       </c>
     </row>
     <row r="25">
@@ -1614,46 +1614,46 @@
         <v>46156.23958333334</v>
       </c>
       <c r="B25" t="n">
-        <v>272</v>
+        <v>328</v>
       </c>
       <c r="C25" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>-126</v>
+        <v>-144</v>
       </c>
       <c r="F25" t="n">
         <v>-2</v>
       </c>
       <c r="G25" t="n">
-        <v>-331</v>
+        <v>-382</v>
       </c>
       <c r="H25" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="I25" t="n">
-        <v>167</v>
+        <v>127</v>
       </c>
       <c r="J25" t="n">
-        <v>97</v>
+        <v>-106</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>-113</v>
+        <v>-130</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>-417</v>
+        <v>-469</v>
       </c>
       <c r="O25" t="n">
-        <v>97</v>
+        <v>-106</v>
       </c>
     </row>
     <row r="26">
@@ -1661,46 +1661,46 @@
         <v>46156.25</v>
       </c>
       <c r="B26" t="n">
-        <v>173</v>
+        <v>290</v>
       </c>
       <c r="C26" t="n">
-        <v>272</v>
+        <v>328</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>-247</v>
+        <v>-273</v>
       </c>
       <c r="F26" t="n">
         <v>-11</v>
       </c>
       <c r="G26" t="n">
-        <v>-99</v>
+        <v>-209</v>
       </c>
       <c r="H26" t="n">
-        <v>272</v>
+        <v>328</v>
       </c>
       <c r="I26" t="n">
-        <v>364</v>
+        <v>466</v>
       </c>
       <c r="J26" t="n">
-        <v>167</v>
+        <v>127</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>-205</v>
+        <v>-233</v>
       </c>
       <c r="M26" t="n">
         <v>-6</v>
       </c>
       <c r="N26" t="n">
-        <v>-305</v>
+        <v>-398</v>
       </c>
       <c r="O26" t="n">
-        <v>167</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27">
@@ -1708,46 +1708,46 @@
         <v>46156.26041666666</v>
       </c>
       <c r="B27" t="n">
-        <v>160</v>
+        <v>203</v>
       </c>
       <c r="C27" t="n">
-        <v>173</v>
+        <v>290</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>-331</v>
+        <v>-382</v>
       </c>
       <c r="F27" t="n">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="G27" t="n">
-        <v>-23</v>
+        <v>-48</v>
       </c>
       <c r="H27" t="n">
-        <v>173</v>
+        <v>290</v>
       </c>
       <c r="I27" t="n">
-        <v>163</v>
+        <v>366</v>
       </c>
       <c r="J27" t="n">
-        <v>364</v>
+        <v>466</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>-417</v>
+        <v>-469</v>
       </c>
       <c r="M27" t="n">
         <v>-21</v>
       </c>
       <c r="N27" t="n">
-        <v>-44</v>
+        <v>-230</v>
       </c>
       <c r="O27" t="n">
-        <v>364</v>
+        <v>466</v>
       </c>
     </row>
     <row r="28">
@@ -1755,46 +1755,46 @@
         <v>46156.27083333334</v>
       </c>
       <c r="B28" t="n">
-        <v>137</v>
+        <v>231</v>
       </c>
       <c r="C28" t="n">
-        <v>160</v>
+        <v>203</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>-99</v>
+        <v>-209</v>
       </c>
       <c r="F28" t="n">
-        <v>-35</v>
+        <v>-40</v>
       </c>
       <c r="G28" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="H28" t="n">
-        <v>160</v>
+        <v>203</v>
       </c>
       <c r="I28" t="n">
-        <v>129</v>
+        <v>360</v>
       </c>
       <c r="J28" t="n">
-        <v>163</v>
+        <v>366</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>-305</v>
+        <v>-398</v>
       </c>
       <c r="M28" t="n">
-        <v>-32</v>
+        <v>-34</v>
       </c>
       <c r="N28" t="n">
-        <v>97</v>
+        <v>-106</v>
       </c>
       <c r="O28" t="n">
-        <v>163</v>
+        <v>366</v>
       </c>
     </row>
     <row r="29">
@@ -1805,43 +1805,43 @@
         <v>94</v>
       </c>
       <c r="C29" t="n">
-        <v>137</v>
+        <v>231</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>-23</v>
+        <v>-48</v>
       </c>
       <c r="F29" t="n">
-        <v>-72</v>
+        <v>-79</v>
       </c>
       <c r="G29" t="n">
-        <v>272</v>
+        <v>328</v>
       </c>
       <c r="H29" t="n">
-        <v>137</v>
+        <v>231</v>
       </c>
       <c r="I29" t="n">
-        <v>282</v>
+        <v>376</v>
       </c>
       <c r="J29" t="n">
-        <v>129</v>
+        <v>360</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>-44</v>
+        <v>-230</v>
       </c>
       <c r="M29" t="n">
-        <v>-59</v>
+        <v>-68</v>
       </c>
       <c r="N29" t="n">
-        <v>167</v>
+        <v>127</v>
       </c>
       <c r="O29" t="n">
-        <v>129</v>
+        <v>360</v>
       </c>
     </row>
     <row r="30">
@@ -1858,13 +1858,13 @@
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="F30" t="n">
-        <v>-126</v>
+        <v>-144</v>
       </c>
       <c r="G30" t="n">
-        <v>173</v>
+        <v>290</v>
       </c>
       <c r="H30" t="n">
         <v>94</v>
@@ -1873,22 +1873,22 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>282</v>
+        <v>376</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>97</v>
+        <v>-106</v>
       </c>
       <c r="M30" t="n">
-        <v>-113</v>
+        <v>-130</v>
       </c>
       <c r="N30" t="n">
-        <v>364</v>
+        <v>466</v>
       </c>
       <c r="O30" t="n">
-        <v>282</v>
+        <v>376</v>
       </c>
     </row>
     <row r="31">
@@ -1905,13 +1905,13 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>272</v>
+        <v>328</v>
       </c>
       <c r="F31" t="n">
-        <v>-247</v>
+        <v>-273</v>
       </c>
       <c r="G31" t="n">
-        <v>160</v>
+        <v>203</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -1926,13 +1926,13 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>167</v>
+        <v>127</v>
       </c>
       <c r="M31" t="n">
-        <v>-205</v>
+        <v>-233</v>
       </c>
       <c r="N31" t="n">
-        <v>163</v>
+        <v>366</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
@@ -1952,13 +1952,13 @@
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>173</v>
+        <v>290</v>
       </c>
       <c r="F32" t="n">
-        <v>-331</v>
+        <v>-382</v>
       </c>
       <c r="G32" t="n">
-        <v>137</v>
+        <v>231</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -1973,13 +1973,13 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>364</v>
+        <v>466</v>
       </c>
       <c r="M32" t="n">
-        <v>-417</v>
+        <v>-469</v>
       </c>
       <c r="N32" t="n">
-        <v>129</v>
+        <v>360</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
@@ -1999,10 +1999,10 @@
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>160</v>
+        <v>203</v>
       </c>
       <c r="F33" t="n">
-        <v>-99</v>
+        <v>-209</v>
       </c>
       <c r="G33" t="n">
         <v>94</v>
@@ -2020,13 +2020,13 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>163</v>
+        <v>366</v>
       </c>
       <c r="M33" t="n">
-        <v>-305</v>
+        <v>-398</v>
       </c>
       <c r="N33" t="n">
-        <v>282</v>
+        <v>376</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
@@ -2046,10 +2046,10 @@
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>137</v>
+        <v>231</v>
       </c>
       <c r="F34" t="n">
-        <v>-23</v>
+        <v>-48</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -2067,10 +2067,10 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>129</v>
+        <v>360</v>
       </c>
       <c r="M34" t="n">
-        <v>-44</v>
+        <v>-230</v>
       </c>
       <c r="N34" t="n">
         <v>0</v>
@@ -2096,7 +2096,7 @@
         <v>94</v>
       </c>
       <c r="F35" t="n">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -2114,10 +2114,10 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>282</v>
+        <v>376</v>
       </c>
       <c r="M35" t="n">
-        <v>97</v>
+        <v>-106</v>
       </c>
       <c r="N35" t="n">
         <v>0</v>
@@ -2143,7 +2143,7 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>272</v>
+        <v>328</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -2164,7 +2164,7 @@
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>167</v>
+        <v>127</v>
       </c>
       <c r="N36" t="n">
         <v>0</v>
@@ -2190,7 +2190,7 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>173</v>
+        <v>290</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -2211,7 +2211,7 @@
         <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>364</v>
+        <v>466</v>
       </c>
       <c r="N37" t="n">
         <v>0</v>
@@ -2237,7 +2237,7 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>160</v>
+        <v>203</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -2258,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>163</v>
+        <v>366</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
@@ -2284,7 +2284,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>137</v>
+        <v>231</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -2305,7 +2305,7 @@
         <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>129</v>
+        <v>360</v>
       </c>
       <c r="N39" t="n">
         <v>0</v>
@@ -2352,7 +2352,7 @@
         <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>282</v>
+        <v>376</v>
       </c>
       <c r="N40" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat: Add impact scale calculations and enhance chart rendering for intraday PAX optimization
</commit_message>
<xml_diff>
--- a/data/simulated_intraday_PAX.xlsx
+++ b/data/simulated_intraday_PAX.xlsx
@@ -1285,7 +1285,7 @@
         <v>46156.16666666666</v>
       </c>
       <c r="B18" t="n">
-        <v>-79</v>
+        <v>-77</v>
       </c>
       <c r="C18" t="n">
         <v>-40</v>
@@ -1332,10 +1332,10 @@
         <v>46156.17708333334</v>
       </c>
       <c r="B19" t="n">
-        <v>-144</v>
+        <v>-139</v>
       </c>
       <c r="C19" t="n">
-        <v>-79</v>
+        <v>-77</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -1350,10 +1350,10 @@
         <v>-11</v>
       </c>
       <c r="H19" t="n">
-        <v>-79</v>
+        <v>-77</v>
       </c>
       <c r="I19" t="n">
-        <v>-130</v>
+        <v>-128</v>
       </c>
       <c r="J19" t="n">
         <v>-68</v>
@@ -1379,10 +1379,10 @@
         <v>46156.1875</v>
       </c>
       <c r="B20" t="n">
-        <v>-273</v>
+        <v>-268</v>
       </c>
       <c r="C20" t="n">
-        <v>-144</v>
+        <v>-139</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -1397,13 +1397,13 @@
         <v>-24</v>
       </c>
       <c r="H20" t="n">
-        <v>-144</v>
+        <v>-139</v>
       </c>
       <c r="I20" t="n">
-        <v>-233</v>
+        <v>-228</v>
       </c>
       <c r="J20" t="n">
-        <v>-130</v>
+        <v>-128</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1418,7 +1418,7 @@
         <v>-21</v>
       </c>
       <c r="O20" t="n">
-        <v>-130</v>
+        <v>-128</v>
       </c>
     </row>
     <row r="21">
@@ -1426,10 +1426,10 @@
         <v>46156.19791666666</v>
       </c>
       <c r="B21" t="n">
-        <v>-382</v>
+        <v>-369</v>
       </c>
       <c r="C21" t="n">
-        <v>-273</v>
+        <v>-268</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -1444,13 +1444,13 @@
         <v>-40</v>
       </c>
       <c r="H21" t="n">
-        <v>-273</v>
+        <v>-268</v>
       </c>
       <c r="I21" t="n">
-        <v>-469</v>
+        <v>-464</v>
       </c>
       <c r="J21" t="n">
-        <v>-233</v>
+        <v>-228</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1465,7 +1465,7 @@
         <v>-34</v>
       </c>
       <c r="O21" t="n">
-        <v>-233</v>
+        <v>-228</v>
       </c>
     </row>
     <row r="22">
@@ -1473,10 +1473,10 @@
         <v>46156.20833333334</v>
       </c>
       <c r="B22" t="n">
-        <v>-209</v>
+        <v>-188</v>
       </c>
       <c r="C22" t="n">
-        <v>-382</v>
+        <v>-369</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -1488,16 +1488,16 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>-79</v>
+        <v>-77</v>
       </c>
       <c r="H22" t="n">
-        <v>-382</v>
+        <v>-369</v>
       </c>
       <c r="I22" t="n">
-        <v>-398</v>
+        <v>-385</v>
       </c>
       <c r="J22" t="n">
-        <v>-469</v>
+        <v>-464</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1512,7 +1512,7 @@
         <v>-68</v>
       </c>
       <c r="O22" t="n">
-        <v>-469</v>
+        <v>-464</v>
       </c>
     </row>
     <row r="23">
@@ -1520,10 +1520,10 @@
         <v>46156.21875</v>
       </c>
       <c r="B23" t="n">
-        <v>-48</v>
+        <v>-10</v>
       </c>
       <c r="C23" t="n">
-        <v>-209</v>
+        <v>-188</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -1535,16 +1535,16 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>-144</v>
+        <v>-139</v>
       </c>
       <c r="H23" t="n">
+        <v>-188</v>
+      </c>
+      <c r="I23" t="n">
         <v>-209</v>
       </c>
-      <c r="I23" t="n">
-        <v>-230</v>
-      </c>
       <c r="J23" t="n">
-        <v>-398</v>
+        <v>-385</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1556,10 +1556,10 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>-130</v>
+        <v>-128</v>
       </c>
       <c r="O23" t="n">
-        <v>-398</v>
+        <v>-385</v>
       </c>
     </row>
     <row r="24">
@@ -1567,31 +1567,31 @@
         <v>46156.22916666666</v>
       </c>
       <c r="B24" t="n">
-        <v>66</v>
+        <v>155</v>
       </c>
       <c r="C24" t="n">
-        <v>-48</v>
+        <v>-10</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>-79</v>
+        <v>-77</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>-273</v>
+        <v>-268</v>
       </c>
       <c r="H24" t="n">
-        <v>-48</v>
+        <v>-10</v>
       </c>
       <c r="I24" t="n">
-        <v>-106</v>
+        <v>-68</v>
       </c>
       <c r="J24" t="n">
-        <v>-230</v>
+        <v>-209</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1603,10 +1603,10 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>-233</v>
+        <v>-228</v>
       </c>
       <c r="O24" t="n">
-        <v>-230</v>
+        <v>-209</v>
       </c>
     </row>
     <row r="25">
@@ -1614,46 +1614,46 @@
         <v>46156.23958333334</v>
       </c>
       <c r="B25" t="n">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="C25" t="n">
-        <v>66</v>
+        <v>155</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>-144</v>
+        <v>-139</v>
       </c>
       <c r="F25" t="n">
         <v>-2</v>
       </c>
       <c r="G25" t="n">
-        <v>-382</v>
+        <v>-369</v>
       </c>
       <c r="H25" t="n">
-        <v>66</v>
+        <v>155</v>
       </c>
       <c r="I25" t="n">
-        <v>127</v>
+        <v>216</v>
       </c>
       <c r="J25" t="n">
-        <v>-106</v>
+        <v>-68</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>-130</v>
+        <v>-128</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>-469</v>
+        <v>-464</v>
       </c>
       <c r="O25" t="n">
-        <v>-106</v>
+        <v>-68</v>
       </c>
     </row>
     <row r="26">
@@ -1661,46 +1661,46 @@
         <v>46156.25</v>
       </c>
       <c r="B26" t="n">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="C26" t="n">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>-273</v>
+        <v>-268</v>
       </c>
       <c r="F26" t="n">
         <v>-11</v>
       </c>
       <c r="G26" t="n">
-        <v>-209</v>
+        <v>-188</v>
       </c>
       <c r="H26" t="n">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="I26" t="n">
-        <v>466</v>
+        <v>453</v>
       </c>
       <c r="J26" t="n">
-        <v>127</v>
+        <v>216</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>-233</v>
+        <v>-228</v>
       </c>
       <c r="M26" t="n">
         <v>-6</v>
       </c>
       <c r="N26" t="n">
-        <v>-398</v>
+        <v>-385</v>
       </c>
       <c r="O26" t="n">
-        <v>127</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27">
@@ -1708,46 +1708,46 @@
         <v>46156.26041666666</v>
       </c>
       <c r="B27" t="n">
-        <v>203</v>
+        <v>160</v>
       </c>
       <c r="C27" t="n">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>-382</v>
+        <v>-369</v>
       </c>
       <c r="F27" t="n">
         <v>-24</v>
       </c>
       <c r="G27" t="n">
-        <v>-48</v>
+        <v>-10</v>
       </c>
       <c r="H27" t="n">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="I27" t="n">
-        <v>366</v>
+        <v>343</v>
       </c>
       <c r="J27" t="n">
-        <v>466</v>
+        <v>453</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>-469</v>
+        <v>-464</v>
       </c>
       <c r="M27" t="n">
         <v>-21</v>
       </c>
       <c r="N27" t="n">
-        <v>-230</v>
+        <v>-209</v>
       </c>
       <c r="O27" t="n">
-        <v>466</v>
+        <v>453</v>
       </c>
     </row>
     <row r="28">
@@ -1755,46 +1755,46 @@
         <v>46156.27083333334</v>
       </c>
       <c r="B28" t="n">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="C28" t="n">
-        <v>203</v>
+        <v>160</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>-209</v>
+        <v>-188</v>
       </c>
       <c r="F28" t="n">
         <v>-40</v>
       </c>
       <c r="G28" t="n">
-        <v>66</v>
+        <v>155</v>
       </c>
       <c r="H28" t="n">
-        <v>203</v>
+        <v>160</v>
       </c>
       <c r="I28" t="n">
-        <v>360</v>
+        <v>317</v>
       </c>
       <c r="J28" t="n">
-        <v>366</v>
+        <v>343</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>-398</v>
+        <v>-385</v>
       </c>
       <c r="M28" t="n">
         <v>-34</v>
       </c>
       <c r="N28" t="n">
-        <v>-106</v>
+        <v>-68</v>
       </c>
       <c r="O28" t="n">
-        <v>366</v>
+        <v>343</v>
       </c>
     </row>
     <row r="29">
@@ -1805,43 +1805,43 @@
         <v>94</v>
       </c>
       <c r="C29" t="n">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>-48</v>
+        <v>-10</v>
       </c>
       <c r="F29" t="n">
-        <v>-79</v>
+        <v>-77</v>
       </c>
       <c r="G29" t="n">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="H29" t="n">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="I29" t="n">
-        <v>376</v>
+        <v>282</v>
       </c>
       <c r="J29" t="n">
-        <v>360</v>
+        <v>317</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>-230</v>
+        <v>-209</v>
       </c>
       <c r="M29" t="n">
         <v>-68</v>
       </c>
       <c r="N29" t="n">
-        <v>127</v>
+        <v>216</v>
       </c>
       <c r="O29" t="n">
-        <v>360</v>
+        <v>317</v>
       </c>
     </row>
     <row r="30">
@@ -1858,13 +1858,13 @@
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>66</v>
+        <v>155</v>
       </c>
       <c r="F30" t="n">
-        <v>-144</v>
+        <v>-139</v>
       </c>
       <c r="G30" t="n">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="H30" t="n">
         <v>94</v>
@@ -1873,22 +1873,22 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>376</v>
+        <v>282</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>-106</v>
+        <v>-68</v>
       </c>
       <c r="M30" t="n">
-        <v>-130</v>
+        <v>-128</v>
       </c>
       <c r="N30" t="n">
-        <v>466</v>
+        <v>453</v>
       </c>
       <c r="O30" t="n">
-        <v>376</v>
+        <v>282</v>
       </c>
     </row>
     <row r="31">
@@ -1905,13 +1905,13 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="F31" t="n">
-        <v>-273</v>
+        <v>-268</v>
       </c>
       <c r="G31" t="n">
-        <v>203</v>
+        <v>160</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -1926,13 +1926,13 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>127</v>
+        <v>216</v>
       </c>
       <c r="M31" t="n">
-        <v>-233</v>
+        <v>-228</v>
       </c>
       <c r="N31" t="n">
-        <v>366</v>
+        <v>343</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
@@ -1952,13 +1952,13 @@
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="F32" t="n">
-        <v>-382</v>
+        <v>-369</v>
       </c>
       <c r="G32" t="n">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -1973,13 +1973,13 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>466</v>
+        <v>453</v>
       </c>
       <c r="M32" t="n">
-        <v>-469</v>
+        <v>-464</v>
       </c>
       <c r="N32" t="n">
-        <v>360</v>
+        <v>317</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
@@ -1999,10 +1999,10 @@
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>203</v>
+        <v>160</v>
       </c>
       <c r="F33" t="n">
-        <v>-209</v>
+        <v>-188</v>
       </c>
       <c r="G33" t="n">
         <v>94</v>
@@ -2020,13 +2020,13 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>366</v>
+        <v>343</v>
       </c>
       <c r="M33" t="n">
-        <v>-398</v>
+        <v>-385</v>
       </c>
       <c r="N33" t="n">
-        <v>376</v>
+        <v>282</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
@@ -2046,10 +2046,10 @@
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="F34" t="n">
-        <v>-48</v>
+        <v>-10</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -2067,10 +2067,10 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>360</v>
+        <v>317</v>
       </c>
       <c r="M34" t="n">
-        <v>-230</v>
+        <v>-209</v>
       </c>
       <c r="N34" t="n">
         <v>0</v>
@@ -2096,7 +2096,7 @@
         <v>94</v>
       </c>
       <c r="F35" t="n">
-        <v>66</v>
+        <v>155</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -2114,10 +2114,10 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>376</v>
+        <v>282</v>
       </c>
       <c r="M35" t="n">
-        <v>-106</v>
+        <v>-68</v>
       </c>
       <c r="N35" t="n">
         <v>0</v>
@@ -2143,7 +2143,7 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -2164,7 +2164,7 @@
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>127</v>
+        <v>216</v>
       </c>
       <c r="N36" t="n">
         <v>0</v>
@@ -2190,7 +2190,7 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -2211,7 +2211,7 @@
         <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>466</v>
+        <v>453</v>
       </c>
       <c r="N37" t="n">
         <v>0</v>
@@ -2237,7 +2237,7 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>203</v>
+        <v>160</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -2258,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>366</v>
+        <v>343</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
@@ -2284,7 +2284,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -2305,7 +2305,7 @@
         <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>360</v>
+        <v>317</v>
       </c>
       <c r="N39" t="n">
         <v>0</v>
@@ -2352,7 +2352,7 @@
         <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>376</v>
+        <v>282</v>
       </c>
       <c r="N40" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Implemented Intraday simulation flight delay
</commit_message>
<xml_diff>
--- a/data/simulated_intraday_PAX.xlsx
+++ b/data/simulated_intraday_PAX.xlsx
@@ -1097,7 +1097,7 @@
         <v>46156.125</v>
       </c>
       <c r="B14" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
@@ -1144,10 +1144,10 @@
         <v>46156.13541666666</v>
       </c>
       <c r="B15" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -1162,10 +1162,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -1191,10 +1191,10 @@
         <v>46156.14583333334</v>
       </c>
       <c r="B16" t="n">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -1209,13 +1209,13 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1230,7 +1230,7 @@
         <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>-6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1238,10 +1238,10 @@
         <v>46156.15625</v>
       </c>
       <c r="B17" t="n">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -1256,13 +1256,13 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>-34</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1277,7 +1277,7 @@
         <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>-21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1285,10 +1285,10 @@
         <v>46156.16666666666</v>
       </c>
       <c r="B18" t="n">
-        <v>-77</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -1300,16 +1300,16 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>-34</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>-34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1332,10 +1332,10 @@
         <v>46156.17708333334</v>
       </c>
       <c r="B19" t="n">
-        <v>-139</v>
+        <v>-2</v>
       </c>
       <c r="C19" t="n">
-        <v>-77</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -1347,16 +1347,16 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>-77</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>-128</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1368,10 +1368,10 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1379,31 +1379,31 @@
         <v>46156.1875</v>
       </c>
       <c r="B20" t="n">
-        <v>-268</v>
+        <v>-5</v>
       </c>
       <c r="C20" t="n">
-        <v>-139</v>
+        <v>-2</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
       <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
         <v>-2</v>
       </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
-        <v>-24</v>
-      </c>
-      <c r="H20" t="n">
-        <v>-139</v>
-      </c>
       <c r="I20" t="n">
-        <v>-228</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>-128</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1415,10 +1415,10 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>-128</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1426,46 +1426,46 @@
         <v>46156.19791666666</v>
       </c>
       <c r="B21" t="n">
-        <v>-369</v>
+        <v>-5</v>
       </c>
       <c r="C21" t="n">
-        <v>-268</v>
+        <v>-5</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>-268</v>
+        <v>-5</v>
       </c>
       <c r="I21" t="n">
-        <v>-464</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>-228</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>-34</v>
+        <v>0</v>
       </c>
       <c r="O21" t="n">
-        <v>-228</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1473,46 +1473,46 @@
         <v>46156.20833333334</v>
       </c>
       <c r="B22" t="n">
-        <v>-188</v>
+        <v>-13</v>
       </c>
       <c r="C22" t="n">
-        <v>-369</v>
+        <v>-5</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>-77</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>-369</v>
+        <v>-5</v>
       </c>
       <c r="I22" t="n">
-        <v>-385</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>-464</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="O22" t="n">
-        <v>-464</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1520,46 +1520,46 @@
         <v>46156.21875</v>
       </c>
       <c r="B23" t="n">
-        <v>-10</v>
+        <v>-21</v>
       </c>
       <c r="C23" t="n">
-        <v>-188</v>
+        <v>-13</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>-139</v>
+        <v>-2</v>
       </c>
       <c r="H23" t="n">
-        <v>-188</v>
+        <v>-13</v>
       </c>
       <c r="I23" t="n">
-        <v>-209</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>-385</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>-34</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>-128</v>
+        <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>-385</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1567,46 +1567,46 @@
         <v>46156.22916666666</v>
       </c>
       <c r="B24" t="n">
-        <v>155</v>
+        <v>-38</v>
       </c>
       <c r="C24" t="n">
-        <v>-10</v>
+        <v>-21</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>-77</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>-268</v>
+        <v>-5</v>
       </c>
       <c r="H24" t="n">
-        <v>-10</v>
+        <v>-21</v>
       </c>
       <c r="I24" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>-209</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>-228</v>
+        <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>-209</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1614,46 +1614,46 @@
         <v>46156.23958333334</v>
       </c>
       <c r="B25" t="n">
-        <v>315</v>
+        <v>-89</v>
       </c>
       <c r="C25" t="n">
-        <v>155</v>
+        <v>-38</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>-139</v>
+        <v>-2</v>
       </c>
       <c r="F25" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>-369</v>
+        <v>-5</v>
       </c>
       <c r="H25" t="n">
-        <v>155</v>
+        <v>-38</v>
       </c>
       <c r="I25" t="n">
-        <v>216</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>-128</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>-464</v>
+        <v>0</v>
       </c>
       <c r="O25" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1661,46 +1661,46 @@
         <v>46156.25</v>
       </c>
       <c r="B26" t="n">
-        <v>267</v>
+        <v>13</v>
       </c>
       <c r="C26" t="n">
-        <v>315</v>
+        <v>-89</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>-268</v>
+        <v>-5</v>
       </c>
       <c r="F26" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>-188</v>
+        <v>-13</v>
       </c>
       <c r="H26" t="n">
-        <v>315</v>
+        <v>-89</v>
       </c>
       <c r="I26" t="n">
-        <v>453</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>216</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>-228</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>-385</v>
+        <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>216</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1708,46 +1708,46 @@
         <v>46156.26041666666</v>
       </c>
       <c r="B27" t="n">
-        <v>160</v>
+        <v>23</v>
       </c>
       <c r="C27" t="n">
-        <v>267</v>
+        <v>13</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>-369</v>
+        <v>-5</v>
       </c>
       <c r="F27" t="n">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>-10</v>
+        <v>-21</v>
       </c>
       <c r="H27" t="n">
-        <v>267</v>
+        <v>13</v>
       </c>
       <c r="I27" t="n">
-        <v>343</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>453</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>-464</v>
+        <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>-209</v>
+        <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1755,46 +1755,46 @@
         <v>46156.27083333334</v>
       </c>
       <c r="B28" t="n">
-        <v>137</v>
+        <v>43</v>
       </c>
       <c r="C28" t="n">
-        <v>160</v>
+        <v>23</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>-188</v>
+        <v>-13</v>
       </c>
       <c r="F28" t="n">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>155</v>
+        <v>-38</v>
       </c>
       <c r="H28" t="n">
-        <v>160</v>
+        <v>23</v>
       </c>
       <c r="I28" t="n">
-        <v>317</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>343</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>-385</v>
+        <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>-34</v>
+        <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>343</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1805,43 +1805,43 @@
         <v>94</v>
       </c>
       <c r="C29" t="n">
-        <v>137</v>
+        <v>43</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>-10</v>
+        <v>-21</v>
       </c>
       <c r="F29" t="n">
-        <v>-77</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>315</v>
+        <v>-89</v>
       </c>
       <c r="H29" t="n">
-        <v>137</v>
+        <v>43</v>
       </c>
       <c r="I29" t="n">
-        <v>282</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>317</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>-209</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>216</v>
+        <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>317</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1858,13 +1858,13 @@
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>155</v>
+        <v>-38</v>
       </c>
       <c r="F30" t="n">
-        <v>-139</v>
+        <v>-2</v>
       </c>
       <c r="G30" t="n">
-        <v>267</v>
+        <v>13</v>
       </c>
       <c r="H30" t="n">
         <v>94</v>
@@ -1873,22 +1873,22 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>282</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>-128</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>453</v>
+        <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>282</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1905,13 +1905,13 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>315</v>
+        <v>-89</v>
       </c>
       <c r="F31" t="n">
-        <v>-268</v>
+        <v>-5</v>
       </c>
       <c r="G31" t="n">
-        <v>160</v>
+        <v>23</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -1926,13 +1926,13 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>216</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>-228</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>343</v>
+        <v>0</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
@@ -1952,13 +1952,13 @@
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>267</v>
+        <v>13</v>
       </c>
       <c r="F32" t="n">
-        <v>-369</v>
+        <v>-5</v>
       </c>
       <c r="G32" t="n">
-        <v>137</v>
+        <v>43</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -1973,13 +1973,13 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>453</v>
+        <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>-464</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>317</v>
+        <v>0</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
@@ -1999,10 +1999,10 @@
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>160</v>
+        <v>23</v>
       </c>
       <c r="F33" t="n">
-        <v>-188</v>
+        <v>-13</v>
       </c>
       <c r="G33" t="n">
         <v>94</v>
@@ -2020,13 +2020,13 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>343</v>
+        <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>-385</v>
+        <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>282</v>
+        <v>0</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
@@ -2046,10 +2046,10 @@
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>137</v>
+        <v>43</v>
       </c>
       <c r="F34" t="n">
-        <v>-10</v>
+        <v>-21</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -2067,10 +2067,10 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>317</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>-209</v>
+        <v>0</v>
       </c>
       <c r="N34" t="n">
         <v>0</v>
@@ -2096,7 +2096,7 @@
         <v>94</v>
       </c>
       <c r="F35" t="n">
-        <v>155</v>
+        <v>-38</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -2114,10 +2114,10 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>282</v>
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="N35" t="n">
         <v>0</v>
@@ -2143,7 +2143,7 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>315</v>
+        <v>-89</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -2164,7 +2164,7 @@
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>216</v>
+        <v>0</v>
       </c>
       <c r="N36" t="n">
         <v>0</v>
@@ -2190,7 +2190,7 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>267</v>
+        <v>13</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -2211,7 +2211,7 @@
         <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>453</v>
+        <v>0</v>
       </c>
       <c r="N37" t="n">
         <v>0</v>
@@ -2237,7 +2237,7 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>160</v>
+        <v>23</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -2258,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>343</v>
+        <v>0</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
@@ -2284,7 +2284,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>137</v>
+        <v>43</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -2305,7 +2305,7 @@
         <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>317</v>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
         <v>0</v>
@@ -2352,7 +2352,7 @@
         <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>282</v>
+        <v>0</v>
       </c>
       <c r="N40" t="n">
         <v>0</v>
@@ -5051,7 +5051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D187"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5088,10 +5088,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>210</v>
+        <v>270</v>
       </c>
       <c r="D2" t="n">
-        <v>225</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3">
@@ -5106,10 +5106,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>225</v>
+        <v>285</v>
       </c>
       <c r="D3" t="n">
-        <v>240</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4">
@@ -5124,10 +5124,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="D4" t="n">
-        <v>255</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5">
@@ -5142,10 +5142,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>255</v>
+        <v>315</v>
       </c>
       <c r="D5" t="n">
-        <v>270</v>
+        <v>330</v>
       </c>
     </row>
     <row r="6">
@@ -5160,10 +5160,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>270</v>
+        <v>330</v>
       </c>
       <c r="D6" t="n">
-        <v>285</v>
+        <v>345</v>
       </c>
     </row>
     <row r="7">
@@ -5178,10 +5178,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>285</v>
+        <v>345</v>
       </c>
       <c r="D7" t="n">
-        <v>300</v>
+        <v>360</v>
       </c>
     </row>
     <row r="8">
@@ -5196,10 +5196,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>300</v>
+        <v>360</v>
       </c>
       <c r="D8" t="n">
-        <v>315</v>
+        <v>375</v>
       </c>
     </row>
     <row r="9">
@@ -5214,10 +5214,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>315</v>
+        <v>375</v>
       </c>
       <c r="D9" t="n">
-        <v>330</v>
+        <v>390</v>
       </c>
     </row>
     <row r="10">
@@ -5232,10 +5232,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>330</v>
+        <v>390</v>
       </c>
       <c r="D10" t="n">
-        <v>345</v>
+        <v>405</v>
       </c>
     </row>
     <row r="11">
@@ -5250,10 +5250,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>345</v>
+        <v>405</v>
       </c>
       <c r="D11" t="n">
-        <v>360</v>
+        <v>420</v>
       </c>
     </row>
     <row r="12">
@@ -5268,10 +5268,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>360</v>
+        <v>420</v>
       </c>
       <c r="D12" t="n">
-        <v>375</v>
+        <v>435</v>
       </c>
     </row>
     <row r="13">
@@ -5282,14 +5282,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>T1_Baggage</t>
+          <t>T1_Boarding</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>375</v>
+        <v>420</v>
       </c>
       <c r="D13" t="n">
-        <v>390</v>
+        <v>435</v>
       </c>
     </row>
     <row r="14">
@@ -5300,14 +5300,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>T1_Baggage</t>
+          <t>T1_Boarding</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>390</v>
+        <v>435</v>
       </c>
       <c r="D14" t="n">
-        <v>405</v>
+        <v>450</v>
       </c>
     </row>
     <row r="15">
@@ -5318,14 +5318,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>T1_Baggage</t>
+          <t>T1_Boarding</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>405</v>
+        <v>450</v>
       </c>
       <c r="D15" t="n">
-        <v>420</v>
+        <v>465</v>
       </c>
     </row>
     <row r="16">
@@ -5336,14 +5336,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>T1_Baggage</t>
+          <t>T1_Boarding</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>420</v>
+        <v>465</v>
       </c>
       <c r="D16" t="n">
-        <v>435</v>
+        <v>480</v>
       </c>
     </row>
     <row r="17">
@@ -5354,14 +5354,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>T1_Baggage</t>
+          <t>T1_Boarding</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>195</v>
+        <v>480</v>
       </c>
       <c r="D17" t="n">
-        <v>210</v>
+        <v>495</v>
       </c>
     </row>
     <row r="18">
@@ -5376,10 +5376,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>360</v>
+        <v>495</v>
       </c>
       <c r="D18" t="n">
-        <v>375</v>
+        <v>510</v>
       </c>
     </row>
     <row r="19">
@@ -5394,10 +5394,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>375</v>
+        <v>510</v>
       </c>
       <c r="D19" t="n">
-        <v>390</v>
+        <v>525</v>
       </c>
     </row>
     <row r="20">
@@ -5412,10 +5412,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>390</v>
+        <v>525</v>
       </c>
       <c r="D20" t="n">
-        <v>405</v>
+        <v>540</v>
       </c>
     </row>
     <row r="21">
@@ -5430,10 +5430,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>405</v>
+        <v>540</v>
       </c>
       <c r="D21" t="n">
-        <v>420</v>
+        <v>555</v>
       </c>
     </row>
     <row r="22">
@@ -5448,10 +5448,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>420</v>
+        <v>555</v>
       </c>
       <c r="D22" t="n">
-        <v>435</v>
+        <v>570</v>
       </c>
     </row>
     <row r="23">
@@ -5466,10 +5466,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>435</v>
+        <v>570</v>
       </c>
       <c r="D23" t="n">
-        <v>450</v>
+        <v>585</v>
       </c>
     </row>
     <row r="24">
@@ -5480,14 +5480,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Checkin</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>450</v>
+        <v>255</v>
       </c>
       <c r="D24" t="n">
-        <v>465</v>
+        <v>270</v>
       </c>
     </row>
     <row r="25">
@@ -5498,14 +5498,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Checkin</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>465</v>
+        <v>270</v>
       </c>
       <c r="D25" t="n">
-        <v>480</v>
+        <v>285</v>
       </c>
     </row>
     <row r="26">
@@ -5516,14 +5516,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Checkin</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>480</v>
+        <v>285</v>
       </c>
       <c r="D26" t="n">
-        <v>495</v>
+        <v>300</v>
       </c>
     </row>
     <row r="27">
@@ -5534,14 +5534,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Checkin</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>495</v>
+        <v>300</v>
       </c>
       <c r="D27" t="n">
-        <v>510</v>
+        <v>315</v>
       </c>
     </row>
     <row r="28">
@@ -5552,14 +5552,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Checkin</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>510</v>
+        <v>315</v>
       </c>
       <c r="D28" t="n">
-        <v>525</v>
+        <v>330</v>
       </c>
     </row>
     <row r="29">
@@ -5570,14 +5570,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Checkin</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>525</v>
+        <v>330</v>
       </c>
       <c r="D29" t="n">
-        <v>540</v>
+        <v>345</v>
       </c>
     </row>
     <row r="30">
@@ -5588,14 +5588,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Checkin</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>540</v>
+        <v>345</v>
       </c>
       <c r="D30" t="n">
-        <v>555</v>
+        <v>360</v>
       </c>
     </row>
     <row r="31">
@@ -5606,14 +5606,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Checkin</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>555</v>
+        <v>360</v>
       </c>
       <c r="D31" t="n">
-        <v>570</v>
+        <v>375</v>
       </c>
     </row>
     <row r="32">
@@ -5624,14 +5624,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Checkin</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>570</v>
+        <v>375</v>
       </c>
       <c r="D32" t="n">
-        <v>585</v>
+        <v>390</v>
       </c>
     </row>
     <row r="33">
@@ -5642,14 +5642,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>T1_Boarding</t>
+          <t>T1_Checkin</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>345</v>
+        <v>390</v>
       </c>
       <c r="D33" t="n">
-        <v>360</v>
+        <v>405</v>
       </c>
     </row>
     <row r="34">
@@ -5664,10 +5664,10 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>195</v>
+        <v>405</v>
       </c>
       <c r="D34" t="n">
-        <v>210</v>
+        <v>420</v>
       </c>
     </row>
     <row r="35">
@@ -5678,14 +5678,14 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>210</v>
+        <v>315</v>
       </c>
       <c r="D35" t="n">
-        <v>225</v>
+        <v>330</v>
       </c>
     </row>
     <row r="36">
@@ -5696,14 +5696,14 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>225</v>
+        <v>330</v>
       </c>
       <c r="D36" t="n">
-        <v>240</v>
+        <v>345</v>
       </c>
     </row>
     <row r="37">
@@ -5714,14 +5714,14 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>240</v>
+        <v>345</v>
       </c>
       <c r="D37" t="n">
-        <v>255</v>
+        <v>360</v>
       </c>
     </row>
     <row r="38">
@@ -5732,14 +5732,14 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>255</v>
+        <v>360</v>
       </c>
       <c r="D38" t="n">
-        <v>270</v>
+        <v>375</v>
       </c>
     </row>
     <row r="39">
@@ -5750,14 +5750,14 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>270</v>
+        <v>375</v>
       </c>
       <c r="D39" t="n">
-        <v>285</v>
+        <v>390</v>
       </c>
     </row>
     <row r="40">
@@ -5768,14 +5768,14 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>285</v>
+        <v>390</v>
       </c>
       <c r="D40" t="n">
-        <v>300</v>
+        <v>405</v>
       </c>
     </row>
     <row r="41">
@@ -5786,14 +5786,14 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>300</v>
+        <v>405</v>
       </c>
       <c r="D41" t="n">
-        <v>315</v>
+        <v>420</v>
       </c>
     </row>
     <row r="42">
@@ -5804,14 +5804,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>315</v>
+        <v>420</v>
       </c>
       <c r="D42" t="n">
-        <v>330</v>
+        <v>435</v>
       </c>
     </row>
     <row r="43">
@@ -5822,14 +5822,14 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>330</v>
+        <v>435</v>
       </c>
       <c r="D43" t="n">
-        <v>345</v>
+        <v>450</v>
       </c>
     </row>
     <row r="44">
@@ -5840,14 +5840,14 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>345</v>
+        <v>450</v>
       </c>
       <c r="D44" t="n">
-        <v>360</v>
+        <v>465</v>
       </c>
     </row>
     <row r="45">
@@ -5858,14 +5858,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Immigration</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>360</v>
+        <v>465</v>
       </c>
       <c r="D45" t="n">
-        <v>375</v>
+        <v>480</v>
       </c>
     </row>
     <row r="46">
@@ -5876,14 +5876,14 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>375</v>
+        <v>345</v>
       </c>
       <c r="D46" t="n">
-        <v>390</v>
+        <v>360</v>
       </c>
     </row>
     <row r="47">
@@ -5894,14 +5894,14 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>390</v>
+        <v>360</v>
       </c>
       <c r="D47" t="n">
-        <v>405</v>
+        <v>375</v>
       </c>
     </row>
     <row r="48">
@@ -5912,14 +5912,14 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>405</v>
+        <v>375</v>
       </c>
       <c r="D48" t="n">
-        <v>420</v>
+        <v>390</v>
       </c>
     </row>
     <row r="49">
@@ -5930,14 +5930,14 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>T1_Checkin</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>180</v>
+        <v>390</v>
       </c>
       <c r="D49" t="n">
-        <v>195</v>
+        <v>405</v>
       </c>
     </row>
     <row r="50">
@@ -5948,14 +5948,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>255</v>
+        <v>405</v>
       </c>
       <c r="D50" t="n">
-        <v>270</v>
+        <v>420</v>
       </c>
     </row>
     <row r="51">
@@ -5966,14 +5966,14 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>270</v>
+        <v>420</v>
       </c>
       <c r="D51" t="n">
-        <v>285</v>
+        <v>435</v>
       </c>
     </row>
     <row r="52">
@@ -5984,14 +5984,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>285</v>
+        <v>435</v>
       </c>
       <c r="D52" t="n">
-        <v>300</v>
+        <v>450</v>
       </c>
     </row>
     <row r="53">
@@ -6002,14 +6002,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="D53" t="n">
-        <v>315</v>
+        <v>465</v>
       </c>
     </row>
     <row r="54">
@@ -6020,14 +6020,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>315</v>
+        <v>465</v>
       </c>
       <c r="D54" t="n">
-        <v>330</v>
+        <v>480</v>
       </c>
     </row>
     <row r="55">
@@ -6038,14 +6038,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>330</v>
+        <v>480</v>
       </c>
       <c r="D55" t="n">
-        <v>345</v>
+        <v>495</v>
       </c>
     </row>
     <row r="56">
@@ -6056,14 +6056,14 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Lounge</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>345</v>
+        <v>495</v>
       </c>
       <c r="D56" t="n">
-        <v>360</v>
+        <v>510</v>
       </c>
     </row>
     <row r="57">
@@ -6074,14 +6074,14 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>360</v>
+        <v>270</v>
       </c>
       <c r="D57" t="n">
-        <v>375</v>
+        <v>285</v>
       </c>
     </row>
     <row r="58">
@@ -6092,14 +6092,14 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>375</v>
+        <v>285</v>
       </c>
       <c r="D58" t="n">
-        <v>390</v>
+        <v>300</v>
       </c>
     </row>
     <row r="59">
@@ -6110,14 +6110,14 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>390</v>
+        <v>300</v>
       </c>
       <c r="D59" t="n">
-        <v>405</v>
+        <v>315</v>
       </c>
     </row>
     <row r="60">
@@ -6128,14 +6128,14 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>405</v>
+        <v>315</v>
       </c>
       <c r="D60" t="n">
-        <v>420</v>
+        <v>330</v>
       </c>
     </row>
     <row r="61">
@@ -6146,14 +6146,14 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>420</v>
+        <v>330</v>
       </c>
       <c r="D61" t="n">
-        <v>435</v>
+        <v>345</v>
       </c>
     </row>
     <row r="62">
@@ -6164,14 +6164,14 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>435</v>
+        <v>345</v>
       </c>
       <c r="D62" t="n">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="63">
@@ -6182,14 +6182,14 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>450</v>
+        <v>360</v>
       </c>
       <c r="D63" t="n">
-        <v>465</v>
+        <v>375</v>
       </c>
     </row>
     <row r="64">
@@ -6200,14 +6200,14 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>465</v>
+        <v>375</v>
       </c>
       <c r="D64" t="n">
-        <v>480</v>
+        <v>390</v>
       </c>
     </row>
     <row r="65">
@@ -6218,14 +6218,14 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>T1_Immigration</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>240</v>
+        <v>390</v>
       </c>
       <c r="D65" t="n">
-        <v>255</v>
+        <v>405</v>
       </c>
     </row>
     <row r="66">
@@ -6236,14 +6236,14 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>T1_Lounge</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>285</v>
+        <v>405</v>
       </c>
       <c r="D66" t="n">
-        <v>300</v>
+        <v>420</v>
       </c>
     </row>
     <row r="67">
@@ -6254,2173 +6254,13 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>T1_Lounge</t>
+          <t>T1_Security</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>300</v>
+        <v>420</v>
       </c>
       <c r="D67" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>315</v>
-      </c>
-      <c r="D68" t="n">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C69" t="n">
-        <v>330</v>
-      </c>
-      <c r="D69" t="n">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
-        <v>345</v>
-      </c>
-      <c r="D70" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C71" t="n">
-        <v>360</v>
-      </c>
-      <c r="D71" t="n">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C72" t="n">
-        <v>375</v>
-      </c>
-      <c r="D72" t="n">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C73" t="n">
-        <v>390</v>
-      </c>
-      <c r="D73" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C74" t="n">
-        <v>405</v>
-      </c>
-      <c r="D74" t="n">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C75" t="n">
-        <v>420</v>
-      </c>
-      <c r="D75" t="n">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C76" t="n">
-        <v>435</v>
-      </c>
-      <c r="D76" t="n">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C77" t="n">
-        <v>450</v>
-      </c>
-      <c r="D77" t="n">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C78" t="n">
-        <v>465</v>
-      </c>
-      <c r="D78" t="n">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C79" t="n">
-        <v>480</v>
-      </c>
-      <c r="D79" t="n">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C80" t="n">
-        <v>495</v>
-      </c>
-      <c r="D80" t="n">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>T1_Lounge</t>
-        </is>
-      </c>
-      <c r="C81" t="n">
-        <v>270</v>
-      </c>
-      <c r="D81" t="n">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C82" t="n">
-        <v>210</v>
-      </c>
-      <c r="D82" t="n">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C83" t="n">
-        <v>225</v>
-      </c>
-      <c r="D83" t="n">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C84" t="n">
-        <v>240</v>
-      </c>
-      <c r="D84" t="n">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C85" t="n">
-        <v>255</v>
-      </c>
-      <c r="D85" t="n">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C86" t="n">
-        <v>270</v>
-      </c>
-      <c r="D86" t="n">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C87" t="n">
-        <v>285</v>
-      </c>
-      <c r="D87" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C88" t="n">
-        <v>300</v>
-      </c>
-      <c r="D88" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C89" t="n">
-        <v>315</v>
-      </c>
-      <c r="D89" t="n">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C90" t="n">
-        <v>330</v>
-      </c>
-      <c r="D90" t="n">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C91" t="n">
-        <v>345</v>
-      </c>
-      <c r="D91" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C92" t="n">
-        <v>360</v>
-      </c>
-      <c r="D92" t="n">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C93" t="n">
-        <v>375</v>
-      </c>
-      <c r="D93" t="n">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C94" t="n">
-        <v>390</v>
-      </c>
-      <c r="D94" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C95" t="n">
-        <v>405</v>
-      </c>
-      <c r="D95" t="n">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C96" t="n">
-        <v>420</v>
-      </c>
-      <c r="D96" t="n">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>T1_Security</t>
-        </is>
-      </c>
-      <c r="C97" t="n">
-        <v>195</v>
-      </c>
-      <c r="D97" t="n">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C98" t="n">
-        <v>210</v>
-      </c>
-      <c r="D98" t="n">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C99" t="n">
-        <v>225</v>
-      </c>
-      <c r="D99" t="n">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C100" t="n">
-        <v>240</v>
-      </c>
-      <c r="D100" t="n">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C101" t="n">
-        <v>255</v>
-      </c>
-      <c r="D101" t="n">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C102" t="n">
-        <v>270</v>
-      </c>
-      <c r="D102" t="n">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C103" t="n">
-        <v>285</v>
-      </c>
-      <c r="D103" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C104" t="n">
-        <v>300</v>
-      </c>
-      <c r="D104" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C105" t="n">
-        <v>315</v>
-      </c>
-      <c r="D105" t="n">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C106" t="n">
-        <v>330</v>
-      </c>
-      <c r="D106" t="n">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C107" t="n">
-        <v>345</v>
-      </c>
-      <c r="D107" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C108" t="n">
-        <v>360</v>
-      </c>
-      <c r="D108" t="n">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C109" t="n">
-        <v>375</v>
-      </c>
-      <c r="D109" t="n">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C110" t="n">
-        <v>390</v>
-      </c>
-      <c r="D110" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C111" t="n">
-        <v>405</v>
-      </c>
-      <c r="D111" t="n">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>T2_Baggage</t>
-        </is>
-      </c>
-      <c r="C112" t="n">
-        <v>420</v>
-      </c>
-      <c r="D112" t="n">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C113" t="n">
-        <v>360</v>
-      </c>
-      <c r="D113" t="n">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C114" t="n">
-        <v>375</v>
-      </c>
-      <c r="D114" t="n">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C115" t="n">
-        <v>390</v>
-      </c>
-      <c r="D115" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C116" t="n">
-        <v>405</v>
-      </c>
-      <c r="D116" t="n">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C117" t="n">
-        <v>420</v>
-      </c>
-      <c r="D117" t="n">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C118" t="n">
-        <v>435</v>
-      </c>
-      <c r="D118" t="n">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C119" t="n">
-        <v>450</v>
-      </c>
-      <c r="D119" t="n">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C120" t="n">
-        <v>465</v>
-      </c>
-      <c r="D120" t="n">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C121" t="n">
-        <v>480</v>
-      </c>
-      <c r="D121" t="n">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C122" t="n">
-        <v>495</v>
-      </c>
-      <c r="D122" t="n">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C123" t="n">
-        <v>510</v>
-      </c>
-      <c r="D123" t="n">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C124" t="n">
-        <v>525</v>
-      </c>
-      <c r="D124" t="n">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C125" t="n">
-        <v>540</v>
-      </c>
-      <c r="D125" t="n">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C126" t="n">
-        <v>555</v>
-      </c>
-      <c r="D126" t="n">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>T2_Boarding</t>
-        </is>
-      </c>
-      <c r="C127" t="n">
-        <v>570</v>
-      </c>
-      <c r="D127" t="n">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C128" t="n">
-        <v>195</v>
-      </c>
-      <c r="D128" t="n">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C129" t="n">
-        <v>210</v>
-      </c>
-      <c r="D129" t="n">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C130" t="n">
-        <v>225</v>
-      </c>
-      <c r="D130" t="n">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C131" t="n">
-        <v>240</v>
-      </c>
-      <c r="D131" t="n">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C132" t="n">
-        <v>255</v>
-      </c>
-      <c r="D132" t="n">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C133" t="n">
-        <v>270</v>
-      </c>
-      <c r="D133" t="n">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C134" t="n">
-        <v>285</v>
-      </c>
-      <c r="D134" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C135" t="n">
-        <v>300</v>
-      </c>
-      <c r="D135" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C136" t="n">
-        <v>315</v>
-      </c>
-      <c r="D136" t="n">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C137" t="n">
-        <v>330</v>
-      </c>
-      <c r="D137" t="n">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C138" t="n">
-        <v>345</v>
-      </c>
-      <c r="D138" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C139" t="n">
-        <v>360</v>
-      </c>
-      <c r="D139" t="n">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C140" t="n">
-        <v>375</v>
-      </c>
-      <c r="D140" t="n">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C141" t="n">
-        <v>390</v>
-      </c>
-      <c r="D141" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>T2_Checkin</t>
-        </is>
-      </c>
-      <c r="C142" t="n">
-        <v>405</v>
-      </c>
-      <c r="D142" t="n">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C143" t="n">
-        <v>255</v>
-      </c>
-      <c r="D143" t="n">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C144" t="n">
-        <v>270</v>
-      </c>
-      <c r="D144" t="n">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C145" t="n">
-        <v>285</v>
-      </c>
-      <c r="D145" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C146" t="n">
-        <v>300</v>
-      </c>
-      <c r="D146" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C147" t="n">
-        <v>315</v>
-      </c>
-      <c r="D147" t="n">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C148" t="n">
-        <v>330</v>
-      </c>
-      <c r="D148" t="n">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C149" t="n">
-        <v>345</v>
-      </c>
-      <c r="D149" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C150" t="n">
-        <v>360</v>
-      </c>
-      <c r="D150" t="n">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C151" t="n">
-        <v>375</v>
-      </c>
-      <c r="D151" t="n">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C152" t="n">
-        <v>390</v>
-      </c>
-      <c r="D152" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C153" t="n">
-        <v>405</v>
-      </c>
-      <c r="D153" t="n">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C154" t="n">
-        <v>420</v>
-      </c>
-      <c r="D154" t="n">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C155" t="n">
-        <v>435</v>
-      </c>
-      <c r="D155" t="n">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C156" t="n">
-        <v>450</v>
-      </c>
-      <c r="D156" t="n">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>T2_Immigration</t>
-        </is>
-      </c>
-      <c r="C157" t="n">
-        <v>465</v>
-      </c>
-      <c r="D157" t="n">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C158" t="n">
-        <v>285</v>
-      </c>
-      <c r="D158" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C159" t="n">
-        <v>300</v>
-      </c>
-      <c r="D159" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C160" t="n">
-        <v>315</v>
-      </c>
-      <c r="D160" t="n">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C161" t="n">
-        <v>330</v>
-      </c>
-      <c r="D161" t="n">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C162" t="n">
-        <v>345</v>
-      </c>
-      <c r="D162" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C163" t="n">
-        <v>360</v>
-      </c>
-      <c r="D163" t="n">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C164" t="n">
-        <v>375</v>
-      </c>
-      <c r="D164" t="n">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C165" t="n">
-        <v>390</v>
-      </c>
-      <c r="D165" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C166" t="n">
-        <v>405</v>
-      </c>
-      <c r="D166" t="n">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C167" t="n">
-        <v>420</v>
-      </c>
-      <c r="D167" t="n">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C168" t="n">
-        <v>435</v>
-      </c>
-      <c r="D168" t="n">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C169" t="n">
-        <v>450</v>
-      </c>
-      <c r="D169" t="n">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C170" t="n">
-        <v>465</v>
-      </c>
-      <c r="D170" t="n">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C171" t="n">
-        <v>480</v>
-      </c>
-      <c r="D171" t="n">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>T2_Lounge</t>
-        </is>
-      </c>
-      <c r="C172" t="n">
-        <v>495</v>
-      </c>
-      <c r="D172" t="n">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C173" t="n">
-        <v>210</v>
-      </c>
-      <c r="D173" t="n">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C174" t="n">
-        <v>225</v>
-      </c>
-      <c r="D174" t="n">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C175" t="n">
-        <v>240</v>
-      </c>
-      <c r="D175" t="n">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C176" t="n">
-        <v>255</v>
-      </c>
-      <c r="D176" t="n">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C177" t="n">
-        <v>270</v>
-      </c>
-      <c r="D177" t="n">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C178" t="n">
-        <v>285</v>
-      </c>
-      <c r="D178" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C179" t="n">
-        <v>300</v>
-      </c>
-      <c r="D179" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C180" t="n">
-        <v>315</v>
-      </c>
-      <c r="D180" t="n">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C181" t="n">
-        <v>330</v>
-      </c>
-      <c r="D181" t="n">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C182" t="n">
-        <v>345</v>
-      </c>
-      <c r="D182" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C183" t="n">
-        <v>360</v>
-      </c>
-      <c r="D183" t="n">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C184" t="n">
-        <v>375</v>
-      </c>
-      <c r="D184" t="n">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C185" t="n">
-        <v>390</v>
-      </c>
-      <c r="D185" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C186" t="n">
-        <v>405</v>
-      </c>
-      <c r="D186" t="n">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>T2_Security</t>
-        </is>
-      </c>
-      <c r="C187" t="n">
-        <v>420</v>
-      </c>
-      <c r="D187" t="n">
         <v>435</v>
       </c>
     </row>

</xml_diff>